<commit_message>
Fixed auction creation flow and retry logic with status
</commit_message>
<xml_diff>
--- a/test-data/Vdata.xlsx
+++ b/test-data/Vdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Mfcwl Projects\ediig-test\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9162D9D6-0AF0-4A54-8AB6-AFAB368AE86C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A0577CD-8EFD-446E-951B-D39271DE77D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{7136C6DB-F0CC-4C33-9575-655EDF0AB019}"/>
   </bookViews>
@@ -3381,7 +3381,7 @@
         <v>32</v>
       </c>
       <c r="Q30" s="12" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="R30" s="8" t="s">
         <v>66</v>
@@ -3428,7 +3428,7 @@
         <v>32</v>
       </c>
       <c r="Q31" s="12" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="R31" s="8" t="s">
         <v>69</v>
@@ -3475,7 +3475,7 @@
         <v>32</v>
       </c>
       <c r="Q32" s="12" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="R32" s="8" t="s">
         <v>70</v>
@@ -3522,7 +3522,7 @@
         <v>32</v>
       </c>
       <c r="Q33" s="12" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="R33" s="8" t="s">
         <v>71</v>
@@ -3569,7 +3569,7 @@
         <v>32</v>
       </c>
       <c r="Q34" s="12" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="R34" s="8" t="s">
         <v>72</v>
@@ -3616,7 +3616,7 @@
         <v>32</v>
       </c>
       <c r="Q35" s="12" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="R35" s="8" t="s">
         <v>73</v>
@@ -3663,7 +3663,7 @@
         <v>32</v>
       </c>
       <c r="Q36" s="12" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="R36" s="8" t="s">
         <v>74</v>
@@ -3710,7 +3710,7 @@
         <v>32</v>
       </c>
       <c r="Q37" s="12" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="R37" s="8" t="s">
         <v>75</v>
@@ -3757,7 +3757,7 @@
         <v>32</v>
       </c>
       <c r="Q38" s="12" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="R38" s="8" t="s">
         <v>78</v>
@@ -3804,7 +3804,7 @@
         <v>32</v>
       </c>
       <c r="Q39" s="12" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="R39" s="8" t="s">
         <v>80</v>
@@ -3851,7 +3851,7 @@
         <v>32</v>
       </c>
       <c r="Q40" s="12" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="R40" s="8" t="s">
         <v>83</v>
@@ -3898,7 +3898,7 @@
         <v>32</v>
       </c>
       <c r="Q41" s="12" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="R41" s="8" t="s">
         <v>85</v>
@@ -3945,7 +3945,7 @@
         <v>32</v>
       </c>
       <c r="Q42" s="12" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="R42" s="8" t="s">
         <v>86</v>
@@ -3992,7 +3992,7 @@
         <v>32</v>
       </c>
       <c r="Q43" s="12" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="R43" s="8" t="s">
         <v>88</v>
@@ -4039,7 +4039,7 @@
         <v>32</v>
       </c>
       <c r="Q44" s="12" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="R44" s="8" t="s">
         <v>89</v>

</xml_diff>